<commit_message>
Dockerizacion del backend y frontend, arreglo de exportacion de prefiniquitos
</commit_message>
<xml_diff>
--- a/backend/app/templates/excel/plantilla_prefiniquitos.xlsx
+++ b/backend/app/templates/excel/plantilla_prefiniquitos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\plantillas general\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_boletas_de_pago-RengifoLtda\backend\app\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85960258-7874-4E34-B908-5B4C164A1122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49210569-F817-42FD-B5A4-E9FDD8B6F999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5DFB6F6D-B14B-4E80-B42B-B6B61AAAA1CB}"/>
   </bookViews>
@@ -110,10 +110,10 @@
     <t>EMPLEADO</t>
   </si>
   <si>
-    <t>.Decreto Supremo Nº 28699 de 1-May-2006</t>
-  </si>
-  <si>
     <t>En caso de que el empleador incumpla su obligación en el plazo establecido en el presente articulo, pagará una multa en beneficio del trabajador consistente en el 30% del monto total a cancelarse, incluyendo mantenimiento de valor (UFVs)</t>
+  </si>
+  <si>
+    <t>Decreto Supremo Nº 28699 de 1-May-2006</t>
   </si>
 </sst>
 </file>
@@ -254,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -268,110 +268,100 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -385,14 +375,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -874,20 +867,20 @@
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
       <c r="G3" s="5"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -900,74 +893,74 @@
     </row>
     <row r="6" spans="2:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="35"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="28"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="40"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="28"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="40"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="28"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="40"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="15"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="29"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="18"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="32"/>
     </row>
     <row r="14" spans="2:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12"/>
@@ -983,317 +976,269 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="11"/>
-      <c r="C16" s="41" t="s">
+      <c r="C16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="30"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
       <c r="G16" s="5"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="11"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="30"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
       <c r="G17" s="5"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="11"/>
-      <c r="C18" s="41" t="s">
+      <c r="C18" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="47"/>
-      <c r="E18" s="47"/>
-      <c r="F18" s="30"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
       <c r="G18" s="5"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="11"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="30"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="30"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
       <c r="G20" s="5"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="11"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
+      <c r="C21" s="12"/>
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="11"/>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="30"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
       <c r="G22" s="5"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="11"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="30"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
+      <c r="C24" s="12"/>
       <c r="G24" s="5"/>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="11"/>
-      <c r="C25" s="41" t="s">
+      <c r="C25" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="30"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="11"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
+      <c r="C26" s="12"/>
       <c r="G26" s="5"/>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="30"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
       <c r="G27" s="5"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="11"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="30"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
       <c r="G28" s="5"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="11"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
+      <c r="C29" s="12"/>
       <c r="G29" s="5"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="30"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
-      <c r="C31" s="41" t="s">
+      <c r="C31" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
-      <c r="F31" s="30"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
       <c r="G31" s="5"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="11"/>
-      <c r="C32" s="41" t="s">
+      <c r="C32" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="30"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="G32" s="5"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="11"/>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="30"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
       <c r="G33" s="5"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="11"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="36"/>
+      <c r="C34" s="12"/>
+      <c r="G34" s="5"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="11"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="36"/>
+      <c r="C35" s="12"/>
+      <c r="G35" s="5"/>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="11"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="34"/>
+      <c r="C36" s="12"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="14"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B37" s="42"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="12"/>
       <c r="G37" s="5"/>
     </row>
     <row r="38" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="11"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
+      <c r="C38" s="12"/>
       <c r="G38" s="5"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="43"/>
-      <c r="C39" s="40"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="54" t="s">
+      <c r="B39" s="21"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="F39" s="54"/>
-      <c r="G39" s="55"/>
+      <c r="F39" s="48"/>
+      <c r="G39" s="49"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B40" s="52" t="s">
+      <c r="B40" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C40" s="53"/>
-      <c r="D40" s="51"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="23"/>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
       <c r="G40" s="8"/>
     </row>
     <row r="41" spans="2:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B42" s="19" t="s">
+      <c r="B42" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C42" s="44"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
-      <c r="F42" s="44"/>
-      <c r="G42" s="45"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="43"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="43"/>
+      <c r="G42" s="44"/>
     </row>
     <row r="43" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" s="45"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="17"/>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" s="45"/>
+      <c r="D44" s="45"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="17"/>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B45" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="17"/>
+    </row>
+    <row r="46" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="39"/>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B44" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="46"/>
-      <c r="F44" s="38"/>
-      <c r="G44" s="39"/>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B45" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="38"/>
-      <c r="E45" s="38"/>
-      <c r="F45" s="38"/>
-      <c r="G45" s="39"/>
-    </row>
-    <row r="46" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="58" t="s">
-        <v>24</v>
-      </c>
-      <c r="C46" s="49"/>
-      <c r="D46" s="49"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="49"/>
-      <c r="G46" s="50"/>
+      <c r="C46" s="51"/>
+      <c r="D46" s="51"/>
+      <c r="E46" s="51"/>
+      <c r="F46" s="51"/>
+      <c r="G46" s="52"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="48"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
-      <c r="F47" s="49"/>
-      <c r="G47" s="50"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="51"/>
+      <c r="E47" s="51"/>
+      <c r="F47" s="51"/>
+      <c r="G47" s="52"/>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B48" s="48"/>
-      <c r="C48" s="49"/>
-      <c r="D48" s="49"/>
-      <c r="E48" s="49"/>
-      <c r="F48" s="49"/>
-      <c r="G48" s="50"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="51"/>
+      <c r="D48" s="51"/>
+      <c r="E48" s="51"/>
+      <c r="F48" s="51"/>
+      <c r="G48" s="52"/>
     </row>
     <row r="49" spans="2:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="35"/>
-      <c r="F49" s="35"/>
-      <c r="G49" s="36"/>
+      <c r="G49" s="5"/>
     </row>
     <row r="50" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="22" t="s">
+      <c r="E50" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="F50" s="22"/>
-      <c r="G50" s="23"/>
+      <c r="F50" s="41"/>
+      <c r="G50" s="42"/>
     </row>
     <row r="51" spans="2:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="6"/>
@@ -1315,25 +1260,25 @@
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B46:G48"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="E39:G39"/>
     <mergeCell ref="C3:F4"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="E39:G39"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="B13:G13"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>